<commit_message>
Update site content and responsive styles
</commit_message>
<xml_diff>
--- a/webfejlesztes_iranyelvek.xlsx
+++ b/webfejlesztes_iranyelvek.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ikelte-my.sharepoint.com/personal/ayp0es_inf_elte_hu/Documents/School/2. felev/Web/Weboldal/TwiceVault/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{C67D3375-103F-4D08-B4DD-D8A083BC79FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C2A98857-BEC1-4BC7-BB41-960CA6F5AD69}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{C67D3375-103F-4D08-B4DD-D8A083BC79FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9589CD8F-7F24-4F04-A971-3E7E58E1A9AD}"/>
   <bookViews>
-    <workbookView xWindow="75" yWindow="660" windowWidth="22200" windowHeight="15465" activeTab="1" xr2:uid="{1BD8638E-000E-4472-8AE1-C32ECD41C6A4}"/>
+    <workbookView xWindow="75" yWindow="660" windowWidth="28650" windowHeight="15465" activeTab="1" xr2:uid="{1BD8638E-000E-4472-8AE1-C32ECD41C6A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Fedőlap" sheetId="2" r:id="rId1"/>
@@ -654,9 +654,6 @@
     <t>A projekt saját CSS fájlokat használ, amelyek jóval több mint 15 szabályt tartalmaznak, validak, és a Bootstrap stílusaitól külön vannak kezelve.</t>
   </si>
   <si>
-    <t>Az oldalak tartalmasak, van legalább 3 külső hivatkozás, és a szerkezeti linkek relatívak.</t>
-  </si>
-  <si>
     <t>A felsorolt tagek mindegyikére van példa, és a szerkezet szemantikusan rendben van</t>
   </si>
   <si>
@@ -676,6 +673,9 @@
   </si>
   <si>
     <t>K-POP Discord közösségben több felhasználó megnyitotta és használta az oldalt különböző környezetekben, így valós használati visszajelzés érkezett. A felmerült problémákat már javítottam(PL lassú timeline betöltés gyengébb készülékeken).</t>
+  </si>
+  <si>
+    <t>Az oldalak tartalmasak, van legalább 3 külső hivatkozás, és a szerkezeti linkek relatívak. Minden fel van töltve tartalommal, viszont a timeline-on nincs ott az összes album, mert adatbázis létrehozása nélkül, statikus weboldalon rendkívül időigényes lett volna mindet odaírni</t>
   </si>
 </sst>
 </file>
@@ -2932,7 +2932,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="80" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="F8" s="78"/>
       <c r="G8" s="83"/>
@@ -2970,7 +2970,7 @@
         <v>1</v>
       </c>
       <c r="E9" s="81" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F9" s="78"/>
       <c r="G9" s="84"/>
@@ -3676,7 +3676,7 @@
         <v>1</v>
       </c>
       <c r="E29" s="80" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F29" s="78"/>
       <c r="G29" s="83"/>
@@ -3784,7 +3784,7 @@
         <v>1</v>
       </c>
       <c r="E32" s="79" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F32" s="78"/>
       <c r="G32" s="82"/>
@@ -3820,7 +3820,7 @@
         <v>1</v>
       </c>
       <c r="E33" s="80" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F33" s="78"/>
       <c r="G33" s="83"/>
@@ -3856,7 +3856,7 @@
         <v>1</v>
       </c>
       <c r="E34" s="81" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F34" s="78"/>
       <c r="G34" s="84"/>
@@ -3998,7 +3998,7 @@
         <v>1</v>
       </c>
       <c r="E38" s="80" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F38" s="78"/>
       <c r="G38" s="83"/>
@@ -4216,7 +4216,7 @@
         <v>1</v>
       </c>
       <c r="E44" s="80" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F44" s="78"/>
       <c r="G44" s="83"/>

</xml_diff>